<commit_message>
Added full text partial queries, accessible via the $text param on query body.
</commit_message>
<xml_diff>
--- a/test/assets/import_standard.xlsx
+++ b/test/assets/import_standard.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t xml:space="preserve">DENOMINAZIONE</t>
   </si>
@@ -37,16 +37,34 @@
     <t xml:space="preserve">PROVINCIA</t>
   </si>
   <si>
-    <t xml:space="preserve">Nome e cognome Esempio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Via Esempio 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BA</t>
+    <t xml:space="preserve">Carmine Conversano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via Duca degli Abruzzi 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">76123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contatto di Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via Suini 504</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contatto di Test 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via Testi 50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09071</t>
   </si>
 </sst>
 </file>
@@ -177,7 +195,7 @@
   <sheetFormatPr defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
@@ -208,27 +226,43 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="n">
         <v>70031</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>

</xml_diff>

<commit_message>
Finished to implement recipients import from XLSX + tests
</commit_message>
<xml_diff>
--- a/test/assets/import_standard.xlsx
+++ b/test/assets/import_standard.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t xml:space="preserve">DENOMINAZIONE</t>
   </si>
@@ -50,6 +50,15 @@
   </si>
   <si>
     <t xml:space="preserve">BT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silvio Troia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Via Sebastiano 52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acerno</t>
   </si>
   <si>
     <t xml:space="preserve">Contatto di Test</t>
@@ -237,39 +246,46 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>70031</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>9</v>
+      <c r="C3" s="0" t="n">
+        <v>84042</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="C4" s="2" t="n">
+        <v>70031</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>

</xml_diff>